<commit_message>
Add Groups & Budget tab with team roster and per-group budget
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WZy7dLHhGnzbT4xp7nPVJM
</commit_message>
<xml_diff>
--- a/TA_Progress_Tracker_Fall2026.xlsx
+++ b/TA_Progress_Tracker_Fall2026.xlsx
@@ -12,7 +12,8 @@
     <sheet name="Supplies &amp; Orders" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="DO Methods" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Contacts" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Meeting Notes" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Groups &amp; Budget" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Meeting Notes" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="CostAll">'Supplies &amp; Orders'!$I$32</definedName>
@@ -38,6 +39,7 @@
     <definedName name="TopMethod">'DO Methods'!$B$6:$B$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Task Tracker'!$A$4:$L$80</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Task Tracker'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Groups &amp; Budget'!$G$9:$J$61</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -45,7 +47,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="11">
+  <numFmts count="12">
     <numFmt numFmtId="164" formatCode="mmm\ d\,\ yyyy"/>
     <numFmt numFmtId="165" formatCode="0;[Red]\-0;&quot;today&quot;"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
@@ -57,8 +59,9 @@
     <numFmt numFmtId="172" formatCode="0.000000"/>
     <numFmt numFmtId="173" formatCode="0\ &quot;°C&quot;"/>
     <numFmt numFmtId="174" formatCode="\+0.000;\-0.000;0.000"/>
+    <numFmt numFmtId="175" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="33">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -199,8 +202,56 @@
       <color rgb="FFCC0000"/>
       <sz val="16"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00CC0000"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000000FF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -249,8 +300,28 @@
         <bgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CC0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF9E5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00262626"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -317,11 +388,69 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="110">
+  <cellXfs count="128">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="20" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -608,6 +737,38 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="175" fontId="28" fillId="10" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="27" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="30" fillId="12" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -11157,6 +11318,1440 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J61"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" style="81" min="1" max="1"/>
+    <col width="22" customWidth="1" style="81" min="2" max="2"/>
+    <col width="14" customWidth="1" style="81" min="3" max="3"/>
+    <col width="22" customWidth="1" style="81" min="4" max="4"/>
+    <col width="12" customWidth="1" style="81" min="5" max="5"/>
+    <col width="3" customWidth="1" style="81" min="6" max="6"/>
+    <col width="5" customWidth="1" style="81" min="7" max="7"/>
+    <col width="9" customWidth="1" style="81" min="8" max="8"/>
+    <col width="34" customWidth="1" style="81" min="9" max="9"/>
+    <col width="26" customWidth="1" style="81" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="110" t="inlineStr">
+        <is>
+          <t>Groups &amp; Budget — who is in each group</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="111" t="inlineStr">
+        <is>
+          <t>From Team_Assignments_Final – Engineering Design 1. Budget = $ per student × students, capped per group. Blue cells are inputs; the summary updates if you move a student in the roster (column H).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="112" t="inlineStr">
+        <is>
+          <t>Budget rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="113" t="inlineStr">
+        <is>
+          <t>Budget per student ($)</t>
+        </is>
+      </c>
+      <c r="D5" s="114" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="113" t="inlineStr">
+        <is>
+          <t>Maximum per group ($)</t>
+        </is>
+      </c>
+      <c r="D6" s="114" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="112" t="inlineStr">
+        <is>
+          <t>Group summary</t>
+        </is>
+      </c>
+      <c r="G8" s="112" t="inlineStr">
+        <is>
+          <t>Roster — student by group</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="115" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="B9" s="115" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="C9" s="116" t="n"/>
+      <c r="D9" s="115" t="inlineStr">
+        <is>
+          <t>Students</t>
+        </is>
+      </c>
+      <c r="E9" s="115" t="inlineStr">
+        <is>
+          <t>Budget ($)</t>
+        </is>
+      </c>
+      <c r="G9" s="115" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="H9" s="115" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="I9" s="115" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="J9" s="115" t="inlineStr">
+        <is>
+          <t>Student</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="117" t="inlineStr">
+        <is>
+          <t>1A</t>
+        </is>
+      </c>
+      <c r="B10" s="118" t="inlineStr">
+        <is>
+          <t>A — DREAM (methylene blue removal)</t>
+        </is>
+      </c>
+      <c r="C10" s="118" t="n"/>
+      <c r="D10" s="119">
+        <f>SUMPRODUCT(($H$10:$H$61=A10)*1)</f>
+        <v/>
+      </c>
+      <c r="E10" s="120">
+        <f>MIN(D10*$D$5,$D$6)</f>
+        <v/>
+      </c>
+      <c r="G10" s="121" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" s="122" t="inlineStr">
+        <is>
+          <t>1A</t>
+        </is>
+      </c>
+      <c r="I10" s="123" t="inlineStr">
+        <is>
+          <t>A — DREAM (methylene blue removal)</t>
+        </is>
+      </c>
+      <c r="J10" s="123" t="inlineStr">
+        <is>
+          <t>Sonu acharya</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="117" t="inlineStr">
+        <is>
+          <t>2A</t>
+        </is>
+      </c>
+      <c r="B11" s="118" t="inlineStr">
+        <is>
+          <t>A — DREAM (methylene blue removal)</t>
+        </is>
+      </c>
+      <c r="C11" s="118" t="n"/>
+      <c r="D11" s="119">
+        <f>SUMPRODUCT(($H$10:$H$61=A11)*1)</f>
+        <v/>
+      </c>
+      <c r="E11" s="120">
+        <f>MIN(D11*$D$5,$D$6)</f>
+        <v/>
+      </c>
+      <c r="G11" s="121" t="n">
+        <v>2</v>
+      </c>
+      <c r="H11" s="122" t="inlineStr">
+        <is>
+          <t>1A</t>
+        </is>
+      </c>
+      <c r="I11" s="123" t="inlineStr">
+        <is>
+          <t>A — DREAM (methylene blue removal)</t>
+        </is>
+      </c>
+      <c r="J11" s="123" t="inlineStr">
+        <is>
+          <t>Elizabeth Dillah</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="117" t="inlineStr">
+        <is>
+          <t>3A</t>
+        </is>
+      </c>
+      <c r="B12" s="118" t="inlineStr">
+        <is>
+          <t>A — DREAM (methylene blue removal)</t>
+        </is>
+      </c>
+      <c r="C12" s="118" t="n"/>
+      <c r="D12" s="119">
+        <f>SUMPRODUCT(($H$10:$H$61=A12)*1)</f>
+        <v/>
+      </c>
+      <c r="E12" s="120">
+        <f>MIN(D12*$D$5,$D$6)</f>
+        <v/>
+      </c>
+      <c r="G12" s="121" t="n">
+        <v>3</v>
+      </c>
+      <c r="H12" s="122" t="inlineStr">
+        <is>
+          <t>1A</t>
+        </is>
+      </c>
+      <c r="I12" s="123" t="inlineStr">
+        <is>
+          <t>A — DREAM (methylene blue removal)</t>
+        </is>
+      </c>
+      <c r="J12" s="123" t="inlineStr">
+        <is>
+          <t>Macie Perrio</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="117" t="inlineStr">
+        <is>
+          <t>4A</t>
+        </is>
+      </c>
+      <c r="B13" s="118" t="inlineStr">
+        <is>
+          <t>A — DREAM (methylene blue removal)</t>
+        </is>
+      </c>
+      <c r="C13" s="118" t="n"/>
+      <c r="D13" s="119">
+        <f>SUMPRODUCT(($H$10:$H$61=A13)*1)</f>
+        <v/>
+      </c>
+      <c r="E13" s="120">
+        <f>MIN(D13*$D$5,$D$6)</f>
+        <v/>
+      </c>
+      <c r="G13" s="121" t="n">
+        <v>4</v>
+      </c>
+      <c r="H13" s="122" t="inlineStr">
+        <is>
+          <t>1A</t>
+        </is>
+      </c>
+      <c r="I13" s="123" t="inlineStr">
+        <is>
+          <t>A — DREAM (methylene blue removal)</t>
+        </is>
+      </c>
+      <c r="J13" s="123" t="inlineStr">
+        <is>
+          <t>Hayden Albert</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="117" t="inlineStr">
+        <is>
+          <t>5A</t>
+        </is>
+      </c>
+      <c r="B14" s="118" t="inlineStr">
+        <is>
+          <t>A — DREAM (methylene blue removal)</t>
+        </is>
+      </c>
+      <c r="C14" s="118" t="n"/>
+      <c r="D14" s="119">
+        <f>SUMPRODUCT(($H$10:$H$61=A14)*1)</f>
+        <v/>
+      </c>
+      <c r="E14" s="120">
+        <f>MIN(D14*$D$5,$D$6)</f>
+        <v/>
+      </c>
+      <c r="G14" s="121" t="n">
+        <v>5</v>
+      </c>
+      <c r="H14" s="122" t="inlineStr">
+        <is>
+          <t>1A</t>
+        </is>
+      </c>
+      <c r="I14" s="123" t="inlineStr">
+        <is>
+          <t>A — DREAM (methylene blue removal)</t>
+        </is>
+      </c>
+      <c r="J14" s="123" t="inlineStr">
+        <is>
+          <t>Hunter Gates</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="117" t="inlineStr">
+        <is>
+          <t>1B</t>
+        </is>
+      </c>
+      <c r="B15" s="118" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="C15" s="118" t="n"/>
+      <c r="D15" s="119">
+        <f>SUMPRODUCT(($H$10:$H$61=A15)*1)</f>
+        <v/>
+      </c>
+      <c r="E15" s="120">
+        <f>MIN(D15*$D$5,$D$6)</f>
+        <v/>
+      </c>
+      <c r="G15" s="121" t="n">
+        <v>6</v>
+      </c>
+      <c r="H15" s="122" t="inlineStr">
+        <is>
+          <t>2A</t>
+        </is>
+      </c>
+      <c r="I15" s="123" t="inlineStr">
+        <is>
+          <t>A — DREAM (methylene blue removal)</t>
+        </is>
+      </c>
+      <c r="J15" s="123" t="inlineStr">
+        <is>
+          <t>Rachel Holmes</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="117" t="inlineStr">
+        <is>
+          <t>2B</t>
+        </is>
+      </c>
+      <c r="B16" s="118" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="C16" s="118" t="n"/>
+      <c r="D16" s="119">
+        <f>SUMPRODUCT(($H$10:$H$61=A16)*1)</f>
+        <v/>
+      </c>
+      <c r="E16" s="120">
+        <f>MIN(D16*$D$5,$D$6)</f>
+        <v/>
+      </c>
+      <c r="G16" s="121" t="n">
+        <v>7</v>
+      </c>
+      <c r="H16" s="122" t="inlineStr">
+        <is>
+          <t>2A</t>
+        </is>
+      </c>
+      <c r="I16" s="123" t="inlineStr">
+        <is>
+          <t>A — DREAM (methylene blue removal)</t>
+        </is>
+      </c>
+      <c r="J16" s="123" t="inlineStr">
+        <is>
+          <t>Shaman Wildman</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="117" t="inlineStr">
+        <is>
+          <t>3B</t>
+        </is>
+      </c>
+      <c r="B17" s="118" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="C17" s="118" t="n"/>
+      <c r="D17" s="119">
+        <f>SUMPRODUCT(($H$10:$H$61=A17)*1)</f>
+        <v/>
+      </c>
+      <c r="E17" s="120">
+        <f>MIN(D17*$D$5,$D$6)</f>
+        <v/>
+      </c>
+      <c r="G17" s="121" t="n">
+        <v>8</v>
+      </c>
+      <c r="H17" s="122" t="inlineStr">
+        <is>
+          <t>2A</t>
+        </is>
+      </c>
+      <c r="I17" s="123" t="inlineStr">
+        <is>
+          <t>A — DREAM (methylene blue removal)</t>
+        </is>
+      </c>
+      <c r="J17" s="123" t="inlineStr">
+        <is>
+          <t>Trevin Cutrer</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="117" t="inlineStr">
+        <is>
+          <t>4B</t>
+        </is>
+      </c>
+      <c r="B18" s="118" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="C18" s="118" t="n"/>
+      <c r="D18" s="119">
+        <f>SUMPRODUCT(($H$10:$H$61=A18)*1)</f>
+        <v/>
+      </c>
+      <c r="E18" s="120">
+        <f>MIN(D18*$D$5,$D$6)</f>
+        <v/>
+      </c>
+      <c r="G18" s="121" t="n">
+        <v>9</v>
+      </c>
+      <c r="H18" s="122" t="inlineStr">
+        <is>
+          <t>2A</t>
+        </is>
+      </c>
+      <c r="I18" s="123" t="inlineStr">
+        <is>
+          <t>A — DREAM (methylene blue removal)</t>
+        </is>
+      </c>
+      <c r="J18" s="123" t="inlineStr">
+        <is>
+          <t>Noah Rodriguez</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="117" t="inlineStr">
+        <is>
+          <t>5B</t>
+        </is>
+      </c>
+      <c r="B19" s="118" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="C19" s="118" t="n"/>
+      <c r="D19" s="119">
+        <f>SUMPRODUCT(($H$10:$H$61=A19)*1)</f>
+        <v/>
+      </c>
+      <c r="E19" s="120">
+        <f>MIN(D19*$D$5,$D$6)</f>
+        <v/>
+      </c>
+      <c r="G19" s="121" t="n">
+        <v>10</v>
+      </c>
+      <c r="H19" s="122" t="inlineStr">
+        <is>
+          <t>3A</t>
+        </is>
+      </c>
+      <c r="I19" s="123" t="inlineStr">
+        <is>
+          <t>A — DREAM (methylene blue removal)</t>
+        </is>
+      </c>
+      <c r="J19" s="123" t="inlineStr">
+        <is>
+          <t>Mia Cuellar</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="117" t="inlineStr">
+        <is>
+          <t>6B</t>
+        </is>
+      </c>
+      <c r="B20" s="118" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="C20" s="118" t="n"/>
+      <c r="D20" s="119">
+        <f>SUMPRODUCT(($H$10:$H$61=A20)*1)</f>
+        <v/>
+      </c>
+      <c r="E20" s="120">
+        <f>MIN(D20*$D$5,$D$6)</f>
+        <v/>
+      </c>
+      <c r="G20" s="121" t="n">
+        <v>11</v>
+      </c>
+      <c r="H20" s="122" t="inlineStr">
+        <is>
+          <t>3A</t>
+        </is>
+      </c>
+      <c r="I20" s="123" t="inlineStr">
+        <is>
+          <t>A — DREAM (methylene blue removal)</t>
+        </is>
+      </c>
+      <c r="J20" s="123" t="inlineStr">
+        <is>
+          <t>Kara Larsen</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="G21" s="121" t="n">
+        <v>12</v>
+      </c>
+      <c r="H21" s="122" t="inlineStr">
+        <is>
+          <t>3A</t>
+        </is>
+      </c>
+      <c r="I21" s="123" t="inlineStr">
+        <is>
+          <t>A — DREAM (methylene blue removal)</t>
+        </is>
+      </c>
+      <c r="J21" s="123" t="inlineStr">
+        <is>
+          <t>Landon Atkins</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="124" t="inlineStr">
+        <is>
+          <t>Project A — DREAM</t>
+        </is>
+      </c>
+      <c r="D22" s="125">
+        <f>COUNTIF($B$10:$B$20,"A — *")&amp;" groups · "&amp;SUMIF($B$10:$B$20,"A — *",$D$10:$D$20)&amp;" students"</f>
+        <v/>
+      </c>
+      <c r="E22" s="126">
+        <f>SUMIF($B$10:$B$20,"A — *",$E$10:$E$20)</f>
+        <v/>
+      </c>
+      <c r="G22" s="121" t="n">
+        <v>13</v>
+      </c>
+      <c r="H22" s="122" t="inlineStr">
+        <is>
+          <t>3A</t>
+        </is>
+      </c>
+      <c r="I22" s="123" t="inlineStr">
+        <is>
+          <t>A — DREAM (methylene blue removal)</t>
+        </is>
+      </c>
+      <c r="J22" s="123" t="inlineStr">
+        <is>
+          <t>Connor Felux</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="124" t="inlineStr">
+        <is>
+          <t>Project B — BOOST</t>
+        </is>
+      </c>
+      <c r="D23" s="125">
+        <f>COUNTIF($B$10:$B$20,"B — *")&amp;" groups · "&amp;SUMIF($B$10:$B$20,"B — *",$D$10:$D$20)&amp;" students"</f>
+        <v/>
+      </c>
+      <c r="E23" s="126">
+        <f>SUMIF($B$10:$B$20,"B — *",$E$10:$E$20)</f>
+        <v/>
+      </c>
+      <c r="G23" s="121" t="n">
+        <v>14</v>
+      </c>
+      <c r="H23" s="122" t="inlineStr">
+        <is>
+          <t>3A</t>
+        </is>
+      </c>
+      <c r="I23" s="123" t="inlineStr">
+        <is>
+          <t>A — DREAM (methylene blue removal)</t>
+        </is>
+      </c>
+      <c r="J23" s="123" t="inlineStr">
+        <is>
+          <t>Axel Cruz-Hernandez</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="124" t="inlineStr">
+        <is>
+          <t>All groups</t>
+        </is>
+      </c>
+      <c r="D24" s="125">
+        <f>COUNTA($A$10:$A$20)&amp;" groups · "&amp;SUM($D$10:$D$20)&amp;" students"</f>
+        <v/>
+      </c>
+      <c r="E24" s="126">
+        <f>SUM($E$10:$E$20)</f>
+        <v/>
+      </c>
+      <c r="G24" s="121" t="n">
+        <v>15</v>
+      </c>
+      <c r="H24" s="122" t="inlineStr">
+        <is>
+          <t>4A</t>
+        </is>
+      </c>
+      <c r="I24" s="123" t="inlineStr">
+        <is>
+          <t>A — DREAM (methylene blue removal)</t>
+        </is>
+      </c>
+      <c r="J24" s="123" t="inlineStr">
+        <is>
+          <t>Brinda Gayen</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="G25" s="121" t="n">
+        <v>16</v>
+      </c>
+      <c r="H25" s="122" t="inlineStr">
+        <is>
+          <t>4A</t>
+        </is>
+      </c>
+      <c r="I25" s="123" t="inlineStr">
+        <is>
+          <t>A — DREAM (methylene blue removal)</t>
+        </is>
+      </c>
+      <c r="J25" s="123" t="inlineStr">
+        <is>
+          <t>Emmalie Potter</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="127" t="inlineStr">
+        <is>
+          <t>Every group has 4–5 students, so every group reaches the $80 cap.</t>
+        </is>
+      </c>
+      <c r="G26" s="121" t="n">
+        <v>17</v>
+      </c>
+      <c r="H26" s="122" t="inlineStr">
+        <is>
+          <t>4A</t>
+        </is>
+      </c>
+      <c r="I26" s="123" t="inlineStr">
+        <is>
+          <t>A — DREAM (methylene blue removal)</t>
+        </is>
+      </c>
+      <c r="J26" s="123" t="inlineStr">
+        <is>
+          <t>Jeremy Brown</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="G27" s="121" t="n">
+        <v>18</v>
+      </c>
+      <c r="H27" s="122" t="inlineStr">
+        <is>
+          <t>4A</t>
+        </is>
+      </c>
+      <c r="I27" s="123" t="inlineStr">
+        <is>
+          <t>A — DREAM (methylene blue removal)</t>
+        </is>
+      </c>
+      <c r="J27" s="123" t="inlineStr">
+        <is>
+          <t>JD Andrade</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="G28" s="121" t="n">
+        <v>19</v>
+      </c>
+      <c r="H28" s="122" t="inlineStr">
+        <is>
+          <t>4A</t>
+        </is>
+      </c>
+      <c r="I28" s="123" t="inlineStr">
+        <is>
+          <t>A — DREAM (methylene blue removal)</t>
+        </is>
+      </c>
+      <c r="J28" s="123" t="inlineStr">
+        <is>
+          <t>Devin Cuellar</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="G29" s="121" t="n">
+        <v>20</v>
+      </c>
+      <c r="H29" s="122" t="inlineStr">
+        <is>
+          <t>5A</t>
+        </is>
+      </c>
+      <c r="I29" s="123" t="inlineStr">
+        <is>
+          <t>A — DREAM (methylene blue removal)</t>
+        </is>
+      </c>
+      <c r="J29" s="123" t="inlineStr">
+        <is>
+          <t>Aaron Linhart</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="G30" s="121" t="n">
+        <v>21</v>
+      </c>
+      <c r="H30" s="122" t="inlineStr">
+        <is>
+          <t>5A</t>
+        </is>
+      </c>
+      <c r="I30" s="123" t="inlineStr">
+        <is>
+          <t>A — DREAM (methylene blue removal)</t>
+        </is>
+      </c>
+      <c r="J30" s="123" t="inlineStr">
+        <is>
+          <t>Diego Leal</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="G31" s="121" t="n">
+        <v>22</v>
+      </c>
+      <c r="H31" s="122" t="inlineStr">
+        <is>
+          <t>5A</t>
+        </is>
+      </c>
+      <c r="I31" s="123" t="inlineStr">
+        <is>
+          <t>A — DREAM (methylene blue removal)</t>
+        </is>
+      </c>
+      <c r="J31" s="123" t="inlineStr">
+        <is>
+          <t>Angel Camarillo</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="G32" s="121" t="n">
+        <v>23</v>
+      </c>
+      <c r="H32" s="122" t="inlineStr">
+        <is>
+          <t>5A</t>
+        </is>
+      </c>
+      <c r="I32" s="123" t="inlineStr">
+        <is>
+          <t>A — DREAM (methylene blue removal)</t>
+        </is>
+      </c>
+      <c r="J32" s="123" t="inlineStr">
+        <is>
+          <t>Mihal Jacob</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="G33" s="121" t="n">
+        <v>24</v>
+      </c>
+      <c r="H33" s="122" t="inlineStr">
+        <is>
+          <t>5A</t>
+        </is>
+      </c>
+      <c r="I33" s="123" t="inlineStr">
+        <is>
+          <t>A — DREAM (methylene blue removal)</t>
+        </is>
+      </c>
+      <c r="J33" s="123" t="inlineStr">
+        <is>
+          <t>David Abagwe</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="G34" s="121" t="n">
+        <v>25</v>
+      </c>
+      <c r="H34" s="122" t="inlineStr">
+        <is>
+          <t>1B</t>
+        </is>
+      </c>
+      <c r="I34" s="123" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="J34" s="123" t="inlineStr">
+        <is>
+          <t>Gavin Cappel</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="G35" s="121" t="n">
+        <v>26</v>
+      </c>
+      <c r="H35" s="122" t="inlineStr">
+        <is>
+          <t>1B</t>
+        </is>
+      </c>
+      <c r="I35" s="123" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="J35" s="123" t="inlineStr">
+        <is>
+          <t>Eric Calderon</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="G36" s="121" t="n">
+        <v>27</v>
+      </c>
+      <c r="H36" s="122" t="inlineStr">
+        <is>
+          <t>1B</t>
+        </is>
+      </c>
+      <c r="I36" s="123" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="J36" s="123" t="inlineStr">
+        <is>
+          <t>Kayra Rushing</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="G37" s="121" t="n">
+        <v>28</v>
+      </c>
+      <c r="H37" s="122" t="inlineStr">
+        <is>
+          <t>1B</t>
+        </is>
+      </c>
+      <c r="I37" s="123" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="J37" s="123" t="inlineStr">
+        <is>
+          <t>Isabella Juarez</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="G38" s="121" t="n">
+        <v>29</v>
+      </c>
+      <c r="H38" s="122" t="inlineStr">
+        <is>
+          <t>1B</t>
+        </is>
+      </c>
+      <c r="I38" s="123" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="J38" s="123" t="inlineStr">
+        <is>
+          <t>Ryan Borkland</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="G39" s="121" t="n">
+        <v>30</v>
+      </c>
+      <c r="H39" s="122" t="inlineStr">
+        <is>
+          <t>2B</t>
+        </is>
+      </c>
+      <c r="I39" s="123" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="J39" s="123" t="inlineStr">
+        <is>
+          <t>Luke Presa</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="G40" s="121" t="n">
+        <v>31</v>
+      </c>
+      <c r="H40" s="122" t="inlineStr">
+        <is>
+          <t>2B</t>
+        </is>
+      </c>
+      <c r="I40" s="123" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="J40" s="123" t="inlineStr">
+        <is>
+          <t>Benjamin Reyes</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="G41" s="121" t="n">
+        <v>32</v>
+      </c>
+      <c r="H41" s="122" t="inlineStr">
+        <is>
+          <t>2B</t>
+        </is>
+      </c>
+      <c r="I41" s="123" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="J41" s="123" t="inlineStr">
+        <is>
+          <t>Victoria Gaytan</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="G42" s="121" t="n">
+        <v>33</v>
+      </c>
+      <c r="H42" s="122" t="inlineStr">
+        <is>
+          <t>2B</t>
+        </is>
+      </c>
+      <c r="I42" s="123" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="J42" s="123" t="inlineStr">
+        <is>
+          <t>Emily Ickert</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="G43" s="121" t="n">
+        <v>34</v>
+      </c>
+      <c r="H43" s="122" t="inlineStr">
+        <is>
+          <t>2B</t>
+        </is>
+      </c>
+      <c r="I43" s="123" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="J43" s="123" t="inlineStr">
+        <is>
+          <t>Veditha Chelikani</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="G44" s="121" t="n">
+        <v>35</v>
+      </c>
+      <c r="H44" s="122" t="inlineStr">
+        <is>
+          <t>3B</t>
+        </is>
+      </c>
+      <c r="I44" s="123" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="J44" s="123" t="inlineStr">
+        <is>
+          <t>Shawn Kwende</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="G45" s="121" t="n">
+        <v>36</v>
+      </c>
+      <c r="H45" s="122" t="inlineStr">
+        <is>
+          <t>3B</t>
+        </is>
+      </c>
+      <c r="I45" s="123" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="J45" s="123" t="inlineStr">
+        <is>
+          <t>Brooke Salada</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="G46" s="121" t="n">
+        <v>37</v>
+      </c>
+      <c r="H46" s="122" t="inlineStr">
+        <is>
+          <t>3B</t>
+        </is>
+      </c>
+      <c r="I46" s="123" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="J46" s="123" t="inlineStr">
+        <is>
+          <t>Lani Allen</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="G47" s="121" t="n">
+        <v>38</v>
+      </c>
+      <c r="H47" s="122" t="inlineStr">
+        <is>
+          <t>3B</t>
+        </is>
+      </c>
+      <c r="I47" s="123" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="J47" s="123" t="inlineStr">
+        <is>
+          <t>Jack Elsas</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="G48" s="121" t="n">
+        <v>39</v>
+      </c>
+      <c r="H48" s="122" t="inlineStr">
+        <is>
+          <t>3B</t>
+        </is>
+      </c>
+      <c r="I48" s="123" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="J48" s="123" t="inlineStr">
+        <is>
+          <t>Jared O'neal</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="G49" s="121" t="n">
+        <v>40</v>
+      </c>
+      <c r="H49" s="122" t="inlineStr">
+        <is>
+          <t>4B</t>
+        </is>
+      </c>
+      <c r="I49" s="123" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="J49" s="123" t="inlineStr">
+        <is>
+          <t>Roman Romashkin</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="G50" s="121" t="n">
+        <v>41</v>
+      </c>
+      <c r="H50" s="122" t="inlineStr">
+        <is>
+          <t>4B</t>
+        </is>
+      </c>
+      <c r="I50" s="123" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="J50" s="123" t="inlineStr">
+        <is>
+          <t>Ashton Adams</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="G51" s="121" t="n">
+        <v>42</v>
+      </c>
+      <c r="H51" s="122" t="inlineStr">
+        <is>
+          <t>4B</t>
+        </is>
+      </c>
+      <c r="I51" s="123" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="J51" s="123" t="inlineStr">
+        <is>
+          <t>Jocelyn Gonzalez</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="G52" s="121" t="n">
+        <v>43</v>
+      </c>
+      <c r="H52" s="122" t="inlineStr">
+        <is>
+          <t>4B</t>
+        </is>
+      </c>
+      <c r="I52" s="123" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="J52" s="123" t="inlineStr">
+        <is>
+          <t>Jenna Koestler</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="G53" s="121" t="n">
+        <v>44</v>
+      </c>
+      <c r="H53" s="122" t="inlineStr">
+        <is>
+          <t>4B</t>
+        </is>
+      </c>
+      <c r="I53" s="123" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="J53" s="123" t="inlineStr">
+        <is>
+          <t>Michelle Gutierrez</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="G54" s="121" t="n">
+        <v>45</v>
+      </c>
+      <c r="H54" s="122" t="inlineStr">
+        <is>
+          <t>5B</t>
+        </is>
+      </c>
+      <c r="I54" s="123" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="J54" s="123" t="inlineStr">
+        <is>
+          <t>Alyssa Jasso</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="G55" s="121" t="n">
+        <v>46</v>
+      </c>
+      <c r="H55" s="122" t="inlineStr">
+        <is>
+          <t>5B</t>
+        </is>
+      </c>
+      <c r="I55" s="123" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="J55" s="123" t="inlineStr">
+        <is>
+          <t>Brisa Colunga</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="G56" s="121" t="n">
+        <v>47</v>
+      </c>
+      <c r="H56" s="122" t="inlineStr">
+        <is>
+          <t>5B</t>
+        </is>
+      </c>
+      <c r="I56" s="123" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="J56" s="123" t="inlineStr">
+        <is>
+          <t>Valeria Leon</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="G57" s="121" t="n">
+        <v>48</v>
+      </c>
+      <c r="H57" s="122" t="inlineStr">
+        <is>
+          <t>5B</t>
+        </is>
+      </c>
+      <c r="I57" s="123" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="J57" s="123" t="inlineStr">
+        <is>
+          <t>Haylee Senior</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="G58" s="121" t="n">
+        <v>49</v>
+      </c>
+      <c r="H58" s="122" t="inlineStr">
+        <is>
+          <t>6B</t>
+        </is>
+      </c>
+      <c r="I58" s="123" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="J58" s="123" t="inlineStr">
+        <is>
+          <t>Maryam Ka</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="G59" s="121" t="n">
+        <v>50</v>
+      </c>
+      <c r="H59" s="122" t="inlineStr">
+        <is>
+          <t>6B</t>
+        </is>
+      </c>
+      <c r="I59" s="123" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="J59" s="123" t="inlineStr">
+        <is>
+          <t>Daniela Osorio</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="G60" s="121" t="n">
+        <v>51</v>
+      </c>
+      <c r="H60" s="122" t="inlineStr">
+        <is>
+          <t>6B</t>
+        </is>
+      </c>
+      <c r="I60" s="123" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="J60" s="123" t="inlineStr">
+        <is>
+          <t>Yasmine Padilla</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="G61" s="121" t="n">
+        <v>52</v>
+      </c>
+      <c r="H61" s="122" t="inlineStr">
+        <is>
+          <t>6B</t>
+        </is>
+      </c>
+      <c r="I61" s="123" t="inlineStr">
+        <is>
+          <t>B — BOOST (oxygenation)</t>
+        </is>
+      </c>
+      <c r="J61" s="123" t="inlineStr">
+        <is>
+          <t>Hayley Ana Tarin</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="G9:J61"/>
+  <mergeCells count="16">
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B12:C12"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="FF7F7F7F"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>

</xml_diff>

<commit_message>
Keep project groups in a standalone file
Add groups/Project_Groups.xlsx (members + budget per group); remove the
groups tab from the TA tracker and the group edits from the quiz roster.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WZy7dLHhGnzbT4xp7nPVJM
</commit_message>
<xml_diff>
--- a/TA_Progress_Tracker_Fall2026.xlsx
+++ b/TA_Progress_Tracker_Fall2026.xlsx
@@ -12,8 +12,7 @@
     <sheet name="Supplies &amp; Orders" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="DO Methods" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Contacts" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Groups &amp; Budget" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Meeting Notes" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Meeting Notes" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="CostAll">'Supplies &amp; Orders'!$I$32</definedName>
@@ -39,7 +38,6 @@
     <definedName name="TopMethod">'DO Methods'!$B$6:$B$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Task Tracker'!$A$4:$M$80</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Task Tracker'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Groups &amp; Budget'!$G$9:$J$61</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -321,7 +319,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -427,6 +425,17 @@
       <right style="thin">
         <color rgb="00BFBFBF"/>
       </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
       <top style="thin">
         <color rgb="00BFBFBF"/>
       </top>
@@ -11488,1440 +11497,6 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J61"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" style="86" min="1" max="1"/>
-    <col width="22" customWidth="1" style="86" min="2" max="2"/>
-    <col width="14" customWidth="1" style="86" min="3" max="3"/>
-    <col width="22" customWidth="1" style="86" min="4" max="4"/>
-    <col width="12" customWidth="1" style="86" min="5" max="5"/>
-    <col width="3" customWidth="1" style="86" min="6" max="6"/>
-    <col width="5" customWidth="1" style="86" min="7" max="7"/>
-    <col width="9" customWidth="1" style="86" min="8" max="8"/>
-    <col width="34" customWidth="1" style="86" min="9" max="9"/>
-    <col width="26" customWidth="1" style="86" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="112" t="inlineStr">
-        <is>
-          <t>Groups &amp; Budget — who is in each group</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="113" t="inlineStr">
-        <is>
-          <t>From Team_Assignments_Final – Engineering Design 1. Budget = $ per student × students, capped per group. Blue cells are inputs; the summary updates if you move a student in the roster (column H).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="114" t="inlineStr">
-        <is>
-          <t>Budget rule</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="115" t="inlineStr">
-        <is>
-          <t>Budget per student ($)</t>
-        </is>
-      </c>
-      <c r="D5" s="116" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="115" t="inlineStr">
-        <is>
-          <t>Maximum per group ($)</t>
-        </is>
-      </c>
-      <c r="D6" s="116" t="n">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="114" t="inlineStr">
-        <is>
-          <t>Group summary</t>
-        </is>
-      </c>
-      <c r="G8" s="114" t="inlineStr">
-        <is>
-          <t>Roster — student by group</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="117" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="B9" s="117" t="inlineStr">
-        <is>
-          <t>Project</t>
-        </is>
-      </c>
-      <c r="C9" s="118" t="n"/>
-      <c r="D9" s="117" t="inlineStr">
-        <is>
-          <t>Students</t>
-        </is>
-      </c>
-      <c r="E9" s="117" t="inlineStr">
-        <is>
-          <t>Budget ($)</t>
-        </is>
-      </c>
-      <c r="G9" s="117" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="H9" s="117" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="I9" s="117" t="inlineStr">
-        <is>
-          <t>Project</t>
-        </is>
-      </c>
-      <c r="J9" s="117" t="inlineStr">
-        <is>
-          <t>Student</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="119" t="inlineStr">
-        <is>
-          <t>1A</t>
-        </is>
-      </c>
-      <c r="B10" s="120" t="inlineStr">
-        <is>
-          <t>A — DREAM (methylene blue removal)</t>
-        </is>
-      </c>
-      <c r="C10" s="120" t="n"/>
-      <c r="D10" s="121">
-        <f>SUMPRODUCT(($H$10:$H$61=A10)*1)</f>
-        <v/>
-      </c>
-      <c r="E10" s="122">
-        <f>MIN(D10*$D$5,$D$6)</f>
-        <v/>
-      </c>
-      <c r="G10" s="123" t="n">
-        <v>1</v>
-      </c>
-      <c r="H10" s="124" t="inlineStr">
-        <is>
-          <t>1A</t>
-        </is>
-      </c>
-      <c r="I10" s="125" t="inlineStr">
-        <is>
-          <t>A — DREAM (methylene blue removal)</t>
-        </is>
-      </c>
-      <c r="J10" s="125" t="inlineStr">
-        <is>
-          <t>Sonu acharya</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="119" t="inlineStr">
-        <is>
-          <t>2A</t>
-        </is>
-      </c>
-      <c r="B11" s="120" t="inlineStr">
-        <is>
-          <t>A — DREAM (methylene blue removal)</t>
-        </is>
-      </c>
-      <c r="C11" s="120" t="n"/>
-      <c r="D11" s="121">
-        <f>SUMPRODUCT(($H$10:$H$61=A11)*1)</f>
-        <v/>
-      </c>
-      <c r="E11" s="122">
-        <f>MIN(D11*$D$5,$D$6)</f>
-        <v/>
-      </c>
-      <c r="G11" s="123" t="n">
-        <v>2</v>
-      </c>
-      <c r="H11" s="124" t="inlineStr">
-        <is>
-          <t>1A</t>
-        </is>
-      </c>
-      <c r="I11" s="125" t="inlineStr">
-        <is>
-          <t>A — DREAM (methylene blue removal)</t>
-        </is>
-      </c>
-      <c r="J11" s="125" t="inlineStr">
-        <is>
-          <t>Elizabeth Dillah</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="119" t="inlineStr">
-        <is>
-          <t>3A</t>
-        </is>
-      </c>
-      <c r="B12" s="120" t="inlineStr">
-        <is>
-          <t>A — DREAM (methylene blue removal)</t>
-        </is>
-      </c>
-      <c r="C12" s="120" t="n"/>
-      <c r="D12" s="121">
-        <f>SUMPRODUCT(($H$10:$H$61=A12)*1)</f>
-        <v/>
-      </c>
-      <c r="E12" s="122">
-        <f>MIN(D12*$D$5,$D$6)</f>
-        <v/>
-      </c>
-      <c r="G12" s="123" t="n">
-        <v>3</v>
-      </c>
-      <c r="H12" s="124" t="inlineStr">
-        <is>
-          <t>1A</t>
-        </is>
-      </c>
-      <c r="I12" s="125" t="inlineStr">
-        <is>
-          <t>A — DREAM (methylene blue removal)</t>
-        </is>
-      </c>
-      <c r="J12" s="125" t="inlineStr">
-        <is>
-          <t>Macie Perrio</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="119" t="inlineStr">
-        <is>
-          <t>4A</t>
-        </is>
-      </c>
-      <c r="B13" s="120" t="inlineStr">
-        <is>
-          <t>A — DREAM (methylene blue removal)</t>
-        </is>
-      </c>
-      <c r="C13" s="120" t="n"/>
-      <c r="D13" s="121">
-        <f>SUMPRODUCT(($H$10:$H$61=A13)*1)</f>
-        <v/>
-      </c>
-      <c r="E13" s="122">
-        <f>MIN(D13*$D$5,$D$6)</f>
-        <v/>
-      </c>
-      <c r="G13" s="123" t="n">
-        <v>4</v>
-      </c>
-      <c r="H13" s="124" t="inlineStr">
-        <is>
-          <t>1A</t>
-        </is>
-      </c>
-      <c r="I13" s="125" t="inlineStr">
-        <is>
-          <t>A — DREAM (methylene blue removal)</t>
-        </is>
-      </c>
-      <c r="J13" s="125" t="inlineStr">
-        <is>
-          <t>Hayden Albert</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="119" t="inlineStr">
-        <is>
-          <t>5A</t>
-        </is>
-      </c>
-      <c r="B14" s="120" t="inlineStr">
-        <is>
-          <t>A — DREAM (methylene blue removal)</t>
-        </is>
-      </c>
-      <c r="C14" s="120" t="n"/>
-      <c r="D14" s="121">
-        <f>SUMPRODUCT(($H$10:$H$61=A14)*1)</f>
-        <v/>
-      </c>
-      <c r="E14" s="122">
-        <f>MIN(D14*$D$5,$D$6)</f>
-        <v/>
-      </c>
-      <c r="G14" s="123" t="n">
-        <v>5</v>
-      </c>
-      <c r="H14" s="124" t="inlineStr">
-        <is>
-          <t>1A</t>
-        </is>
-      </c>
-      <c r="I14" s="125" t="inlineStr">
-        <is>
-          <t>A — DREAM (methylene blue removal)</t>
-        </is>
-      </c>
-      <c r="J14" s="125" t="inlineStr">
-        <is>
-          <t>Hunter Gates</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="119" t="inlineStr">
-        <is>
-          <t>1B</t>
-        </is>
-      </c>
-      <c r="B15" s="120" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="C15" s="120" t="n"/>
-      <c r="D15" s="121">
-        <f>SUMPRODUCT(($H$10:$H$61=A15)*1)</f>
-        <v/>
-      </c>
-      <c r="E15" s="122">
-        <f>MIN(D15*$D$5,$D$6)</f>
-        <v/>
-      </c>
-      <c r="G15" s="123" t="n">
-        <v>6</v>
-      </c>
-      <c r="H15" s="124" t="inlineStr">
-        <is>
-          <t>2A</t>
-        </is>
-      </c>
-      <c r="I15" s="125" t="inlineStr">
-        <is>
-          <t>A — DREAM (methylene blue removal)</t>
-        </is>
-      </c>
-      <c r="J15" s="125" t="inlineStr">
-        <is>
-          <t>Rachel Holmes</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="119" t="inlineStr">
-        <is>
-          <t>2B</t>
-        </is>
-      </c>
-      <c r="B16" s="120" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="C16" s="120" t="n"/>
-      <c r="D16" s="121">
-        <f>SUMPRODUCT(($H$10:$H$61=A16)*1)</f>
-        <v/>
-      </c>
-      <c r="E16" s="122">
-        <f>MIN(D16*$D$5,$D$6)</f>
-        <v/>
-      </c>
-      <c r="G16" s="123" t="n">
-        <v>7</v>
-      </c>
-      <c r="H16" s="124" t="inlineStr">
-        <is>
-          <t>2A</t>
-        </is>
-      </c>
-      <c r="I16" s="125" t="inlineStr">
-        <is>
-          <t>A — DREAM (methylene blue removal)</t>
-        </is>
-      </c>
-      <c r="J16" s="125" t="inlineStr">
-        <is>
-          <t>Shaman Wildman</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="119" t="inlineStr">
-        <is>
-          <t>3B</t>
-        </is>
-      </c>
-      <c r="B17" s="120" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="C17" s="120" t="n"/>
-      <c r="D17" s="121">
-        <f>SUMPRODUCT(($H$10:$H$61=A17)*1)</f>
-        <v/>
-      </c>
-      <c r="E17" s="122">
-        <f>MIN(D17*$D$5,$D$6)</f>
-        <v/>
-      </c>
-      <c r="G17" s="123" t="n">
-        <v>8</v>
-      </c>
-      <c r="H17" s="124" t="inlineStr">
-        <is>
-          <t>2A</t>
-        </is>
-      </c>
-      <c r="I17" s="125" t="inlineStr">
-        <is>
-          <t>A — DREAM (methylene blue removal)</t>
-        </is>
-      </c>
-      <c r="J17" s="125" t="inlineStr">
-        <is>
-          <t>Trevin Cutrer</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="119" t="inlineStr">
-        <is>
-          <t>4B</t>
-        </is>
-      </c>
-      <c r="B18" s="120" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="C18" s="120" t="n"/>
-      <c r="D18" s="121">
-        <f>SUMPRODUCT(($H$10:$H$61=A18)*1)</f>
-        <v/>
-      </c>
-      <c r="E18" s="122">
-        <f>MIN(D18*$D$5,$D$6)</f>
-        <v/>
-      </c>
-      <c r="G18" s="123" t="n">
-        <v>9</v>
-      </c>
-      <c r="H18" s="124" t="inlineStr">
-        <is>
-          <t>2A</t>
-        </is>
-      </c>
-      <c r="I18" s="125" t="inlineStr">
-        <is>
-          <t>A — DREAM (methylene blue removal)</t>
-        </is>
-      </c>
-      <c r="J18" s="125" t="inlineStr">
-        <is>
-          <t>Noah Rodriguez</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="119" t="inlineStr">
-        <is>
-          <t>5B</t>
-        </is>
-      </c>
-      <c r="B19" s="120" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="C19" s="120" t="n"/>
-      <c r="D19" s="121">
-        <f>SUMPRODUCT(($H$10:$H$61=A19)*1)</f>
-        <v/>
-      </c>
-      <c r="E19" s="122">
-        <f>MIN(D19*$D$5,$D$6)</f>
-        <v/>
-      </c>
-      <c r="G19" s="123" t="n">
-        <v>10</v>
-      </c>
-      <c r="H19" s="124" t="inlineStr">
-        <is>
-          <t>3A</t>
-        </is>
-      </c>
-      <c r="I19" s="125" t="inlineStr">
-        <is>
-          <t>A — DREAM (methylene blue removal)</t>
-        </is>
-      </c>
-      <c r="J19" s="125" t="inlineStr">
-        <is>
-          <t>Mia Cuellar</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="119" t="inlineStr">
-        <is>
-          <t>6B</t>
-        </is>
-      </c>
-      <c r="B20" s="120" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="C20" s="120" t="n"/>
-      <c r="D20" s="121">
-        <f>SUMPRODUCT(($H$10:$H$61=A20)*1)</f>
-        <v/>
-      </c>
-      <c r="E20" s="122">
-        <f>MIN(D20*$D$5,$D$6)</f>
-        <v/>
-      </c>
-      <c r="G20" s="123" t="n">
-        <v>11</v>
-      </c>
-      <c r="H20" s="124" t="inlineStr">
-        <is>
-          <t>3A</t>
-        </is>
-      </c>
-      <c r="I20" s="125" t="inlineStr">
-        <is>
-          <t>A — DREAM (methylene blue removal)</t>
-        </is>
-      </c>
-      <c r="J20" s="125" t="inlineStr">
-        <is>
-          <t>Kara Larsen</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="G21" s="123" t="n">
-        <v>12</v>
-      </c>
-      <c r="H21" s="124" t="inlineStr">
-        <is>
-          <t>3A</t>
-        </is>
-      </c>
-      <c r="I21" s="125" t="inlineStr">
-        <is>
-          <t>A — DREAM (methylene blue removal)</t>
-        </is>
-      </c>
-      <c r="J21" s="125" t="inlineStr">
-        <is>
-          <t>Landon Atkins</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="126" t="inlineStr">
-        <is>
-          <t>Project A — DREAM</t>
-        </is>
-      </c>
-      <c r="D22" s="127">
-        <f>COUNTIF($B$10:$B$20,"A — *")&amp;" groups · "&amp;SUMIF($B$10:$B$20,"A — *",$D$10:$D$20)&amp;" students"</f>
-        <v/>
-      </c>
-      <c r="E22" s="128">
-        <f>SUMIF($B$10:$B$20,"A — *",$E$10:$E$20)</f>
-        <v/>
-      </c>
-      <c r="G22" s="123" t="n">
-        <v>13</v>
-      </c>
-      <c r="H22" s="124" t="inlineStr">
-        <is>
-          <t>3A</t>
-        </is>
-      </c>
-      <c r="I22" s="125" t="inlineStr">
-        <is>
-          <t>A — DREAM (methylene blue removal)</t>
-        </is>
-      </c>
-      <c r="J22" s="125" t="inlineStr">
-        <is>
-          <t>Connor Felux</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="126" t="inlineStr">
-        <is>
-          <t>Project B — BOOST</t>
-        </is>
-      </c>
-      <c r="D23" s="127">
-        <f>COUNTIF($B$10:$B$20,"B — *")&amp;" groups · "&amp;SUMIF($B$10:$B$20,"B — *",$D$10:$D$20)&amp;" students"</f>
-        <v/>
-      </c>
-      <c r="E23" s="128">
-        <f>SUMIF($B$10:$B$20,"B — *",$E$10:$E$20)</f>
-        <v/>
-      </c>
-      <c r="G23" s="123" t="n">
-        <v>14</v>
-      </c>
-      <c r="H23" s="124" t="inlineStr">
-        <is>
-          <t>3A</t>
-        </is>
-      </c>
-      <c r="I23" s="125" t="inlineStr">
-        <is>
-          <t>A — DREAM (methylene blue removal)</t>
-        </is>
-      </c>
-      <c r="J23" s="125" t="inlineStr">
-        <is>
-          <t>Axel Cruz-Hernandez</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="126" t="inlineStr">
-        <is>
-          <t>All groups</t>
-        </is>
-      </c>
-      <c r="D24" s="127">
-        <f>COUNTA($A$10:$A$20)&amp;" groups · "&amp;SUM($D$10:$D$20)&amp;" students"</f>
-        <v/>
-      </c>
-      <c r="E24" s="128">
-        <f>SUM($E$10:$E$20)</f>
-        <v/>
-      </c>
-      <c r="G24" s="123" t="n">
-        <v>15</v>
-      </c>
-      <c r="H24" s="124" t="inlineStr">
-        <is>
-          <t>4A</t>
-        </is>
-      </c>
-      <c r="I24" s="125" t="inlineStr">
-        <is>
-          <t>A — DREAM (methylene blue removal)</t>
-        </is>
-      </c>
-      <c r="J24" s="125" t="inlineStr">
-        <is>
-          <t>Brinda Gayen</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="G25" s="123" t="n">
-        <v>16</v>
-      </c>
-      <c r="H25" s="124" t="inlineStr">
-        <is>
-          <t>4A</t>
-        </is>
-      </c>
-      <c r="I25" s="125" t="inlineStr">
-        <is>
-          <t>A — DREAM (methylene blue removal)</t>
-        </is>
-      </c>
-      <c r="J25" s="125" t="inlineStr">
-        <is>
-          <t>Emmalie Potter</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="129" t="inlineStr">
-        <is>
-          <t>Every group has 4–5 students, so every group reaches the $80 cap.</t>
-        </is>
-      </c>
-      <c r="G26" s="123" t="n">
-        <v>17</v>
-      </c>
-      <c r="H26" s="124" t="inlineStr">
-        <is>
-          <t>4A</t>
-        </is>
-      </c>
-      <c r="I26" s="125" t="inlineStr">
-        <is>
-          <t>A — DREAM (methylene blue removal)</t>
-        </is>
-      </c>
-      <c r="J26" s="125" t="inlineStr">
-        <is>
-          <t>Jeremy Brown</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="G27" s="123" t="n">
-        <v>18</v>
-      </c>
-      <c r="H27" s="124" t="inlineStr">
-        <is>
-          <t>4A</t>
-        </is>
-      </c>
-      <c r="I27" s="125" t="inlineStr">
-        <is>
-          <t>A — DREAM (methylene blue removal)</t>
-        </is>
-      </c>
-      <c r="J27" s="125" t="inlineStr">
-        <is>
-          <t>JD Andrade</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="G28" s="123" t="n">
-        <v>19</v>
-      </c>
-      <c r="H28" s="124" t="inlineStr">
-        <is>
-          <t>4A</t>
-        </is>
-      </c>
-      <c r="I28" s="125" t="inlineStr">
-        <is>
-          <t>A — DREAM (methylene blue removal)</t>
-        </is>
-      </c>
-      <c r="J28" s="125" t="inlineStr">
-        <is>
-          <t>Devin Cuellar</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="G29" s="123" t="n">
-        <v>20</v>
-      </c>
-      <c r="H29" s="124" t="inlineStr">
-        <is>
-          <t>5A</t>
-        </is>
-      </c>
-      <c r="I29" s="125" t="inlineStr">
-        <is>
-          <t>A — DREAM (methylene blue removal)</t>
-        </is>
-      </c>
-      <c r="J29" s="125" t="inlineStr">
-        <is>
-          <t>Aaron Linhart</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="G30" s="123" t="n">
-        <v>21</v>
-      </c>
-      <c r="H30" s="124" t="inlineStr">
-        <is>
-          <t>5A</t>
-        </is>
-      </c>
-      <c r="I30" s="125" t="inlineStr">
-        <is>
-          <t>A — DREAM (methylene blue removal)</t>
-        </is>
-      </c>
-      <c r="J30" s="125" t="inlineStr">
-        <is>
-          <t>Diego Leal</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="G31" s="123" t="n">
-        <v>22</v>
-      </c>
-      <c r="H31" s="124" t="inlineStr">
-        <is>
-          <t>5A</t>
-        </is>
-      </c>
-      <c r="I31" s="125" t="inlineStr">
-        <is>
-          <t>A — DREAM (methylene blue removal)</t>
-        </is>
-      </c>
-      <c r="J31" s="125" t="inlineStr">
-        <is>
-          <t>Angel Camarillo</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="G32" s="123" t="n">
-        <v>23</v>
-      </c>
-      <c r="H32" s="124" t="inlineStr">
-        <is>
-          <t>5A</t>
-        </is>
-      </c>
-      <c r="I32" s="125" t="inlineStr">
-        <is>
-          <t>A — DREAM (methylene blue removal)</t>
-        </is>
-      </c>
-      <c r="J32" s="125" t="inlineStr">
-        <is>
-          <t>Mihal Jacob</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="G33" s="123" t="n">
-        <v>24</v>
-      </c>
-      <c r="H33" s="124" t="inlineStr">
-        <is>
-          <t>5A</t>
-        </is>
-      </c>
-      <c r="I33" s="125" t="inlineStr">
-        <is>
-          <t>A — DREAM (methylene blue removal)</t>
-        </is>
-      </c>
-      <c r="J33" s="125" t="inlineStr">
-        <is>
-          <t>David Abagwe</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="G34" s="123" t="n">
-        <v>25</v>
-      </c>
-      <c r="H34" s="124" t="inlineStr">
-        <is>
-          <t>1B</t>
-        </is>
-      </c>
-      <c r="I34" s="125" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="J34" s="125" t="inlineStr">
-        <is>
-          <t>Gavin Cappel</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="G35" s="123" t="n">
-        <v>26</v>
-      </c>
-      <c r="H35" s="124" t="inlineStr">
-        <is>
-          <t>1B</t>
-        </is>
-      </c>
-      <c r="I35" s="125" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="J35" s="125" t="inlineStr">
-        <is>
-          <t>Eric Calderon</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="G36" s="123" t="n">
-        <v>27</v>
-      </c>
-      <c r="H36" s="124" t="inlineStr">
-        <is>
-          <t>1B</t>
-        </is>
-      </c>
-      <c r="I36" s="125" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="J36" s="125" t="inlineStr">
-        <is>
-          <t>Kayra Rushing</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="G37" s="123" t="n">
-        <v>28</v>
-      </c>
-      <c r="H37" s="124" t="inlineStr">
-        <is>
-          <t>1B</t>
-        </is>
-      </c>
-      <c r="I37" s="125" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="J37" s="125" t="inlineStr">
-        <is>
-          <t>Isabella Juarez</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="G38" s="123" t="n">
-        <v>29</v>
-      </c>
-      <c r="H38" s="124" t="inlineStr">
-        <is>
-          <t>1B</t>
-        </is>
-      </c>
-      <c r="I38" s="125" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="J38" s="125" t="inlineStr">
-        <is>
-          <t>Ryan Borkland</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="G39" s="123" t="n">
-        <v>30</v>
-      </c>
-      <c r="H39" s="124" t="inlineStr">
-        <is>
-          <t>2B</t>
-        </is>
-      </c>
-      <c r="I39" s="125" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="J39" s="125" t="inlineStr">
-        <is>
-          <t>Luke Presa</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="G40" s="123" t="n">
-        <v>31</v>
-      </c>
-      <c r="H40" s="124" t="inlineStr">
-        <is>
-          <t>2B</t>
-        </is>
-      </c>
-      <c r="I40" s="125" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="J40" s="125" t="inlineStr">
-        <is>
-          <t>Benjamin Reyes</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="G41" s="123" t="n">
-        <v>32</v>
-      </c>
-      <c r="H41" s="124" t="inlineStr">
-        <is>
-          <t>2B</t>
-        </is>
-      </c>
-      <c r="I41" s="125" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="J41" s="125" t="inlineStr">
-        <is>
-          <t>Victoria Gaytan</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="G42" s="123" t="n">
-        <v>33</v>
-      </c>
-      <c r="H42" s="124" t="inlineStr">
-        <is>
-          <t>2B</t>
-        </is>
-      </c>
-      <c r="I42" s="125" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="J42" s="125" t="inlineStr">
-        <is>
-          <t>Emily Ickert</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="G43" s="123" t="n">
-        <v>34</v>
-      </c>
-      <c r="H43" s="124" t="inlineStr">
-        <is>
-          <t>2B</t>
-        </is>
-      </c>
-      <c r="I43" s="125" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="J43" s="125" t="inlineStr">
-        <is>
-          <t>Veditha Chelikani</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="G44" s="123" t="n">
-        <v>35</v>
-      </c>
-      <c r="H44" s="124" t="inlineStr">
-        <is>
-          <t>3B</t>
-        </is>
-      </c>
-      <c r="I44" s="125" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="J44" s="125" t="inlineStr">
-        <is>
-          <t>Shawn Kwende</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="G45" s="123" t="n">
-        <v>36</v>
-      </c>
-      <c r="H45" s="124" t="inlineStr">
-        <is>
-          <t>3B</t>
-        </is>
-      </c>
-      <c r="I45" s="125" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="J45" s="125" t="inlineStr">
-        <is>
-          <t>Brooke Salada</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="G46" s="123" t="n">
-        <v>37</v>
-      </c>
-      <c r="H46" s="124" t="inlineStr">
-        <is>
-          <t>3B</t>
-        </is>
-      </c>
-      <c r="I46" s="125" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="J46" s="125" t="inlineStr">
-        <is>
-          <t>Lani Allen</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="G47" s="123" t="n">
-        <v>38</v>
-      </c>
-      <c r="H47" s="124" t="inlineStr">
-        <is>
-          <t>3B</t>
-        </is>
-      </c>
-      <c r="I47" s="125" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="J47" s="125" t="inlineStr">
-        <is>
-          <t>Jack Elsas</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="G48" s="123" t="n">
-        <v>39</v>
-      </c>
-      <c r="H48" s="124" t="inlineStr">
-        <is>
-          <t>3B</t>
-        </is>
-      </c>
-      <c r="I48" s="125" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="J48" s="125" t="inlineStr">
-        <is>
-          <t>Jared O'neal</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="G49" s="123" t="n">
-        <v>40</v>
-      </c>
-      <c r="H49" s="124" t="inlineStr">
-        <is>
-          <t>4B</t>
-        </is>
-      </c>
-      <c r="I49" s="125" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="J49" s="125" t="inlineStr">
-        <is>
-          <t>Roman Romashkin</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="G50" s="123" t="n">
-        <v>41</v>
-      </c>
-      <c r="H50" s="124" t="inlineStr">
-        <is>
-          <t>4B</t>
-        </is>
-      </c>
-      <c r="I50" s="125" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="J50" s="125" t="inlineStr">
-        <is>
-          <t>Ashton Adams</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="G51" s="123" t="n">
-        <v>42</v>
-      </c>
-      <c r="H51" s="124" t="inlineStr">
-        <is>
-          <t>4B</t>
-        </is>
-      </c>
-      <c r="I51" s="125" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="J51" s="125" t="inlineStr">
-        <is>
-          <t>Jocelyn Gonzalez</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="G52" s="123" t="n">
-        <v>43</v>
-      </c>
-      <c r="H52" s="124" t="inlineStr">
-        <is>
-          <t>4B</t>
-        </is>
-      </c>
-      <c r="I52" s="125" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="J52" s="125" t="inlineStr">
-        <is>
-          <t>Jenna Koestler</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="G53" s="123" t="n">
-        <v>44</v>
-      </c>
-      <c r="H53" s="124" t="inlineStr">
-        <is>
-          <t>4B</t>
-        </is>
-      </c>
-      <c r="I53" s="125" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="J53" s="125" t="inlineStr">
-        <is>
-          <t>Michelle Gutierrez</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="G54" s="123" t="n">
-        <v>45</v>
-      </c>
-      <c r="H54" s="124" t="inlineStr">
-        <is>
-          <t>5B</t>
-        </is>
-      </c>
-      <c r="I54" s="125" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="J54" s="125" t="inlineStr">
-        <is>
-          <t>Alyssa Jasso</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="G55" s="123" t="n">
-        <v>46</v>
-      </c>
-      <c r="H55" s="124" t="inlineStr">
-        <is>
-          <t>5B</t>
-        </is>
-      </c>
-      <c r="I55" s="125" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="J55" s="125" t="inlineStr">
-        <is>
-          <t>Brisa Colunga</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="G56" s="123" t="n">
-        <v>47</v>
-      </c>
-      <c r="H56" s="124" t="inlineStr">
-        <is>
-          <t>5B</t>
-        </is>
-      </c>
-      <c r="I56" s="125" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="J56" s="125" t="inlineStr">
-        <is>
-          <t>Valeria Leon</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="G57" s="123" t="n">
-        <v>48</v>
-      </c>
-      <c r="H57" s="124" t="inlineStr">
-        <is>
-          <t>5B</t>
-        </is>
-      </c>
-      <c r="I57" s="125" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="J57" s="125" t="inlineStr">
-        <is>
-          <t>Haylee Senior</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="G58" s="123" t="n">
-        <v>49</v>
-      </c>
-      <c r="H58" s="124" t="inlineStr">
-        <is>
-          <t>6B</t>
-        </is>
-      </c>
-      <c r="I58" s="125" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="J58" s="125" t="inlineStr">
-        <is>
-          <t>Maryam Ka</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="G59" s="123" t="n">
-        <v>50</v>
-      </c>
-      <c r="H59" s="124" t="inlineStr">
-        <is>
-          <t>6B</t>
-        </is>
-      </c>
-      <c r="I59" s="125" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="J59" s="125" t="inlineStr">
-        <is>
-          <t>Daniela Osorio</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="G60" s="123" t="n">
-        <v>51</v>
-      </c>
-      <c r="H60" s="124" t="inlineStr">
-        <is>
-          <t>6B</t>
-        </is>
-      </c>
-      <c r="I60" s="125" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="J60" s="125" t="inlineStr">
-        <is>
-          <t>Yasmine Padilla</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="G61" s="123" t="n">
-        <v>52</v>
-      </c>
-      <c r="H61" s="124" t="inlineStr">
-        <is>
-          <t>6B</t>
-        </is>
-      </c>
-      <c r="I61" s="125" t="inlineStr">
-        <is>
-          <t>B — BOOST (oxygenation)</t>
-        </is>
-      </c>
-      <c r="J61" s="125" t="inlineStr">
-        <is>
-          <t>Hayley Ana Tarin</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="G9:J61"/>
-  <mergeCells count="16">
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="A22:C22"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="A24:C24"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B12:C12"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
     <tabColor rgb="FF7F7F7F"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>

</xml_diff>